<commit_message>
Automate Redfin ZIP downloads from official public files
</commit_message>
<xml_diff>
--- a/metadata/docx_variable_audit.xlsx
+++ b/metadata/docx_variable_audit.xlsx
@@ -3726,14 +3726,14 @@
         <v>40939</v>
       </c>
       <c r="Z19" s="1" t="n">
-        <v>46173</v>
+        <v>46265</v>
       </c>
       <c r="AA19" t="n">
-        <v>24391</v>
+        <v>28920</v>
       </c>
       <c r="AB19" t="inlineStr">
         <is>
-          <t>63 missing of 24391 fact rows</t>
+          <t>806 missing of 28920 fact rows</t>
         </is>
       </c>
       <c r="AC19" t="inlineStr">
@@ -4041,14 +4041,14 @@
         <v>40939</v>
       </c>
       <c r="Z22" s="1" t="n">
-        <v>46173</v>
+        <v>46265</v>
       </c>
       <c r="AA22" t="n">
-        <v>24391</v>
+        <v>28920</v>
       </c>
       <c r="AB22" t="inlineStr">
         <is>
-          <t>31 missing of 24391 fact rows</t>
+          <t>563 missing of 28920 fact rows</t>
         </is>
       </c>
       <c r="AC22" t="inlineStr">
@@ -4146,14 +4146,14 @@
         <v>40939</v>
       </c>
       <c r="Z23" s="1" t="n">
-        <v>46173</v>
+        <v>46265</v>
       </c>
       <c r="AA23" t="n">
-        <v>24391</v>
+        <v>28920</v>
       </c>
       <c r="AB23" t="inlineStr">
         <is>
-          <t>63 missing of 24391 fact rows</t>
+          <t>806 missing of 28920 fact rows</t>
         </is>
       </c>
       <c r="AC23" t="inlineStr">
@@ -5188,14 +5188,14 @@
         <v>40939</v>
       </c>
       <c r="Z33" s="1" t="n">
-        <v>46173</v>
+        <v>46265</v>
       </c>
       <c r="AA33" t="n">
-        <v>24391</v>
+        <v>28920</v>
       </c>
       <c r="AB33" t="inlineStr">
         <is>
-          <t>63 missing of 24391 fact rows</t>
+          <t>813 missing of 28920 fact rows</t>
         </is>
       </c>
       <c r="AC33" t="inlineStr">

</xml_diff>